<commit_message>
Capturing latency in the o/p file
</commit_message>
<xml_diff>
--- a/evaluation_results_tp.xlsx
+++ b/evaluation_results_tp.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,21 @@
           <t>raw_response</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>request_time</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>response_time</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>latency_mmss</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -498,29 +513,60 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Error: 500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>RESULT:
+This bar chart illustrates the actual spend to date across different channels.
+**Key insights from the chart:**
+*   The 'Offsite' channel accounts for the highest spend to date.
+*   'Onsite' and 'App' channels also show significant spend, following 'Offsite'.
+*   'In-store' has the lowest actual spend to date among the listed channels.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SELECT
+    t1.channels,
+    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date
+  FROM
+    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1
+  GROUP BY
+    t1.channels
+  LIMIT 500</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"chart_type": null, "x_axis_label": null, "y_axis_label": null}</t>
+          <t>{"chart_type": "bar", "x_axis_label": "Channels", "y_axis_label": "Total Actual Spend To Date ($)"}</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>-0.0379</v>
+        <v>0.878</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>0.9817</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
+          <t>[{"invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"all_db_settings": {"use_database": "BigQuery"}, "database_settings": {"bq_project_id": "acn-cda", "bq_dataset_id": "RMN_Campaign_Dataset_Dev", "bq_ddl_schema": "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", "transpile_to_bigquery": true, "process_input_errors": true, "process_tool_output_errors": true, "number_of_candidates": 1, "model": "gemini-2.5-flash", "temperature": 0.01, "generate_sql_type": "dc"}}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "fbkHNhD8", "timestamp": 1757660031.761983}, {"content": {"parts": [{"functionCall": {"id": "adk-9b83588a-963b-43bc-bd9f-12b8db000970", "args": {"question": "actual spend to date by channel from campaign_performance table"}, "name": "call_db_agent"}}], "role": "model"}, "usageMetadata": {"candidatesTokenCount": 17, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 17}], "promptTokenCount": 8280, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8280}], "thoughtsTokenCount": 173, "totalTokenCount": 8470, "trafficType": "ON_DEMAND"}, "invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "8qO0iVTs", "timestamp": 1757660031.763616}, {"content": {"parts": [{"functionResponse": {"id": "adk-9b83588a-963b-43bc-bd9f-12b8db000970", "name": "call_db_agent", "response": {"result": "```json\n{\n  \"explain\": \"The query calculates the total actual spend to date for each marketing channel by summing the `actual_spend_to_date` column and grouping the results by the `channels` column from the `campaign_performance` table.\",\n  \"sql\": \"SELECT\\n    t1.channels,\\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  GROUP BY\\n    t1.channels\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"channels\": \"Onsite\",\n      \"total_actual_spend_to_date\": 133455139.97500044\n    },\n    {\n      \"channels\": \"App\",\n      \"total_actual_spend_to_date\": 126214368.35499968\n    },\n    {\n      \"channels\": \"Offsite\",\n      \"total_actual_spend_to_date\": 156833302.079999\n    },\n    {\n      \"channels\": \"Channel-CTV\",\n      \"total_actual_spend_to_date\": 46984040.660000049\n    },\n    {\n      \"channels\": \"In-store\",\n      \"total_actual_spend_to_date\": 32660484.865000207\n    }\n  ],\n  \"nl_results\": \"The actual spend to date by channel is as follows:\\n- Onsite: 133,455,139.98\\n- App: 126,214,368.35\\n- Offsite: 156,833,302.08\\n- Channel-CTV: 46,984,040.66\\n- In-store: 32,660,484.87\"\n}\n```"}}}], "role": "user"}, "invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"sql_query": "SELECT\n    t1.channels,\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\n  FROM\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\n  GROUP BY\n    t1.channels\n  LIMIT 500", "query_result": [{"channels": "Onsite", "total_actual_spend_to_date": 133455139.97500044}, {"channels": "App", "total_actual_spend_to_date": 126214368.35499968}, {"channels": "Offsite", "total_actual_spend_to_date": 156833302.079999}, {"channels": "Channel-CTV", "total_actual_spend_to_date": 46984040.66000005}, {"channels": "In-store", "total_actual_spend_to_date": 32660484.865000207}], "db_agent_output": "```json\n{\n  \"explain\": \"The query calculates the total actual spend to date for each marketing channel by summing the `actual_spend_to_date` column and grouping the results by the `channels` column from the `campaign_performance` table.\",\n  \"sql\": \"SELECT\\n    t1.channels,\\n    SUM(t1.actual_spend_to_date) AS total_actual_spend_to_date\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  GROUP BY\\n    t1.channels\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"channels\": \"Onsite\",\n      \"total_actual_spend_to_date\": 133455139.97500044\n    },\n    {\n      \"channels\": \"App\",\n      \"total_actual_spend_to_date\": 126214368.35499968\n    },\n    {\n      \"channels\": \"Offsite\",\n      \"total_actual_spend_to_date\": 156833302.079999\n    },\n    {\n      \"channels\": \"Channel-CTV\",\n      \"total_actual_spend_to_date\": 46984040.660000049\n    },\n    {\n      \"channels\": \"In-store\",\n      \"total_actual_spend_to_date\": 32660484.865000207\n    }\n  ],\n  \"nl_results\": \"The actual spend to date by channel is as follows:\\n- Onsite: 133,455,139.98\\n- App: 126,214,368.35\\n- Offsite: 156,833,302.08\\n- Channel-CTV: 46,984,040.66\\n- In-store: 32,660,484.87\"\n}\n```"}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "vBpjmtFC", "timestamp": 1757660081.685995}, {"content": {"parts": [{"functionCall": {"id": "adk-11189fbf-21ef-4a80-93bf-fe5c3aa886d2", "args": {"question": "bar chart of actual spend to date by channel"}, "name": "call_viz_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7606}], "cachedContentTokenCount": 7606, "candidatesTokenCount": 15, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 15}], "promptTokenCount": 8820, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8820}], "thoughtsTokenCount": 179, "totalTokenCount": 9014, "trafficType": "ON_DEMAND"}, "invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "xU7g41Cn", "timestamp": 1757660081.687622}, {"content": {"parts": [{"functionResponse": {"id": "adk-11189fbf-21ef-4a80-93bf-fe5c3aa886d2", "name": "call_viz_agent", "response": {"text": "This bar chart illustrates the actual spend to date across different channels.\n\n**Key insights from the chart:**\n*   The 'Offsite' channel accounts for the highest spend to date.\n*   'Onsite' and 'App' channels also show significant spend, following 'Offsite'.\n*   'In-store' has the lowest actual spend to date among the listed channels.", "images": []}}}], "role": "user"}, "invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"chart_type": "bar", "x_axis_label": "Channels", "y_axis_label": "Total Actual Spend To Date ($)", "x": [], "y": [], "categories": ["Onsite", "App", "Offsite", "Channel-CTV", "In-store"], "values": [133455139.97500044, 126214368.35499968, 156833302.079999, 46984040.66000005, 32660484.865000207], "title": "Actual Spend to Date by Channel", "stages": [], "subcategories": [], "dv_agent_output": "This bar chart illustrates the actual spend to date across different channels.\n\n**Key insights from the chart:**\n*   The 'Offsite' channel accounts for the highest spend to date.\n*   'Onsite' and 'App' channels also show significant spend, following 'Offsite'.\n*   'In-store' has the lowest actual spend to date among the listed channels."}, "artifactDelta": {"chart_20250912_122500.png": 0}, "requestedAuthConfigs": {}}, "id": "zPuqAjrR", "timestamp": 1757660109.837661}, {"content": {"parts": [{"text": "RESULT:\nThis bar chart illustrates the actual spend to date across different channels.\n\n**Key insights from the chart:**\n*   The 'Offsite' channel accounts for the highest spend to date.\n*   'Onsite' and 'App' channels also show significant spend, following 'Offsite'.\n*   'In-store' has the lowest actual spend to date among the listed channels."}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7584}], "cachedContentTokenCount": 7584, "candidatesTokenCount": 83, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 83}], "promptTokenCount": 8997, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8997}], "thoughtsTokenCount": 125, "totalTokenCount": 9205, "trafficType": "ON_DEMAND"}, "invocationId": "e-8f418de9-d187-4446-b1a8-09228abb78e5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "Magebtvs", "timestamp": 1757660109.839109}]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:53:51.731836Z</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:55:20.803597Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1:29.072</t>
         </is>
       </c>
     </row>
@@ -545,20 +591,56 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Error: 500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>**Result:**
+The total conversions by audience segment are:
+- Cart Abandoners: 175,430
+- Geo-Targeted Shoppers: 148,821
+- Loyalty Program Members: 145,905
+- Frequent Buyers: 142,301
+- Deal Hunters: 141,497
+- Lookalike Audiences: 137,501
+- New to Category: 130,697
+- Promo Responders: 122,216
+- Seasonal Shoppers: 112,235
+- App Engaged Shoppers: 106,473
+- New to Brand: 94,798
+- High-Intent Visitors: 93,765
+- Frequent Browsers: 85,921
+- Brand Interactors: 72,356
+- Category Enthusiasts: 72,173
+- Auto-Replenish Candidates: 47,004
+- Brand Loyalists: 43,964
+- Value Shoppers: 39,209
+- Churn Risk: 38,452
+- Repeat Buyers: 34,849
+A pie chart showing 'Conversions by Audience Segment' has been created. Each slice represents an audience segment, and its size corresponds to the 'total_conversions' for that segment. This chart effectively illustrates the proportion of conversions contributed by different audience segments.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SELECT
+    t2.audience_segment,
+    SUM(t1.conversions) AS total_conversions
+  FROM
+    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1
+    INNER JOIN `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` AS t2 ON t1.audience_id = t2.audience_id
+  GROUP BY
+    t2.audience_segment
+  ORDER BY
+    total_conversions DESC
+  LIMIT 500</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"chart_type": null, "x_axis_label": null, "y_axis_label": null}</t>
+          <t>{"chart_type": "pie", "x_axis_label": null, "y_axis_label": null}</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>-0.0785</v>
+        <v>0.8478</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>0.903</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -567,7 +649,22 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>500 Server Error: Internal Server Error for url: http://127.0.0.1:8000/run</t>
+          <t>[{"invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {"all_db_settings": {"use_database": "BigQuery"}, "database_settings": {"bq_project_id": "acn-cda", "bq_dataset_id": "RMN_Campaign_Dataset_Dev", "bq_ddl_schema": "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", "transpile_to_bigquery": true, "process_input_errors": true, "process_tool_output_errors": true, "number_of_candidates": 1, "model": "gemini-2.5-flash", "temperature": 0.01, "generate_sql_type": "dc"}}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "1URWOD4G", "timestamp": 1757660121.258028}, {"content": {"parts": [{"functionCall": {"id": "adk-3880083d-2e18-46a2-8308-dbbd0cc1bc25", "args": {"question": "conversions by audience segment"}, "name": "call_db_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7610}], "cachedContentTokenCount": 7610, "candidatesTokenCount": 10, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 10}], "promptTokenCount": 8264, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8264}], "thoughtsTokenCount": 164, "totalTokenCount": 8438, "trafficType": "ON_DEMAND"}, "invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "ZrqetoMo", "timestamp": 1757660121.25975}, {"content": {"parts": [{"functionResponse": {"id": "adk-3880083d-2e18-46a2-8308-dbbd0cc1bc25", "name": "call_db_agent", "response": {"result": "```json\n{\n  \"explain\": \"The query joins the `campaign_performance` table (aliased as `t1`) with the `audience_data` table (aliased as `t2`) on the `audience_id` column. It then calculates the sum of `conversions` for each `audience_segment` and orders the results in descending order of total conversions, limiting to the top 500.\",\n  \"sql\": \"SELECT\\n    t2.audience_segment,\\n    SUM(t1.conversions) AS total_conversions\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n    INNER JOIN `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` AS t2 ON t1.audience_id = t2.audience_id\\n  GROUP BY\\n    t2.audience_segment\\n  ORDER BY\\n    total_conversions DESC\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"audience_segment\": \"Cart Abandoners\",\n      \"total_conversions\": 175430\n    },\n    {\n      \"audience_segment\": \"Geo-Targeted Shoppers\",\n      \"total_conversions\": 148821\n    },\n    {\n      \"audience_segment\": \"Loyalty Program Members\",\n      \"total_conversions\": 145905\n    },\n    {\n      \"audience_segment\": \"Frequent Buyers\",\n      \"total_conversions\": 142301\n    },\n    {\n      \"audience_segment\": \"Deal Hunters\",\n      \"total_conversions\": 141497\n    },\n    {\n      \"audience_segment\": \"Lookalike Audiences\",\n      \"total_conversions\": 137501\n    },\n    {\n      \"audience_segment\": \"New to Category\",\n      \"total_conversions\": 130697\n    },\n    {\n      \"audience_segment\": \"Promo Responders\",\n      \"total_conversions\": 122216\n    },\n    {\n      \"audience_segment\": \"Seasonal Shoppers\",\n      \"total_conversions\": 112235\n    },\n    {\n      \"audience_segment\": \"App Engaged Shoppers\",\n      \"total_conversions\": 106473\n    },\n    {\n      \"audience_segment\": \"New to Brand\",\n      \"total_conversions\": 94798\n    },\n    {\n      \"audience_segment\": \"High-Intent Visitors\",\n      \"total_conversions\": 93765\n    },\n    {\n      \"audience_segment\": \"Frequent Browsers\",\n      \"total_conversions\": 85921\n    },\n    {\n      \"audience_segment\": \"Brand Interactors\",\n      \"total_conversions\": 72356\n    },\n    {\n      \"audience_segment\": \"Category Enthusiasts\",\n      \"total_conversions\": 72173\n    },\n    {\n      \"audience_segment\": \"Auto-Replenish Candidates\",\n      \"total_conversions\": 47004\n    },\n    {\n      \"audience_segment\": \"Brand Loyalists\",\n      \"total_conversions\": 43964\n    },\n    {\n      \"audience_segment\": \"Value Shoppers\",\n      \"total_conversions\": 39209\n    },\n    {\n      \"audience_segment\": \"Churn Risk\",\n      \"total_conversions\": 38452\n    },\n    {\n      \"audience_segment\": \"Repeat Buyers\",\n      \"total_conversions\": 34849\n  }],\n  \"nl_results\": \"The total conversions by audience segment are:\\n- Cart Abandoners: 175,430\\n- Geo-Targeted Shoppers: 148,821\\n- Loyalty Program Members: 145,905\\n- Frequent Buyers: 142,301\\n- Deal Hunters: 141,497\\n- Lookalike Audiences: 137,501\\n- New to Category: 130,697\\n- Promo Responders: 122,216\\n- Seasonal Shoppers: 112,235\\n- App Engaged Shoppers: 106,473\\n- New to Brand: 94,798\\n- High-Intent Visitors: 93,765\\n- Frequent Browsers: 85,921\\n- Brand Interactors: 72,356\\n- Category Enthusiasts: 72,173\\n- Auto-Replenish Candidates: 47,004\\n- Brand Loyalists: 43,964\\n- Value Shoppers: 39,209\\n- Churn Risk: 38,452\\n- Repeat Buyers: 34,849\"\n}\n```"}}}], "role": "user"}, "invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {"sql_query": "SELECT\n    t2.audience_segment,\n    SUM(t1.conversions) AS total_conversions\n  FROM\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\n    INNER JOIN `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` AS t2 ON t1.audience_id = t2.audience_id\n  GROUP BY\n    t2.audience_segment\n  ORDER BY\n    total_conversions DESC\n  LIMIT 500", "query_result": [{"audience_segment": "Cart Abandoners", "total_conversions": 175430.0}, {"audience_segment": "Geo-Targeted Shoppers", "total_conversions": 148821.0}, {"audience_segment": "Loyalty Program Members", "total_conversions": 145905.0}, {"audience_segment": "Frequent Buyers", "total_conversions": 142301.0}, {"audience_segment": "Deal Hunters", "total_conversions": 141497.0}, {"audience_segment": "Lookalike Audiences", "total_conversions": 137501.0}, {"audience_segment": "New to Category", "total_conversions": 130697.0}, {"audience_segment": "Promo Responders", "total_conversions": 122216.0}, {"audience_segment": "Seasonal Shoppers", "total_conversions": 112235.0}, {"audience_segment": "App Engaged Shoppers", "total_conversions": 106473.0}, {"audience_segment": "New to Brand", "total_conversions": 94798.0}, {"audience_segment": "High-Intent Visitors", "total_conversions": 93765.0}, {"audience_segment": "Frequent Browsers", "total_conversions": 85921.0}, {"audience_segment": "Brand Interactors", "total_conversions": 72356.0}, {"audience_segment": "Category Enthusiasts", "total_conversions": 72173.0}, {"audience_segment": "Auto-Replenish Candidates", "total_conversions": 47004.0}, {"audience_segment": "Brand Loyalists", "total_conversions": 43964.0}, {"audience_segment": "Value Shoppers", "total_conversions": 39209.0}, {"audience_segment": "Churn Risk", "total_conversions": 38452.0}, {"audience_segment": "Repeat Buyers", "total_conversions": 34849.0}], "db_agent_output": "```json\n{\n  \"explain\": \"The query joins the `campaign_performance` table (aliased as `t1`) with the `audience_data` table (aliased as `t2`) on the `audience_id` column. It then calculates the sum of `conversions` for each `audience_segment` and orders the results in descending order of total conversions, limiting to the top 500.\",\n  \"sql\": \"SELECT\\n    t2.audience_segment,\\n    SUM(t1.conversions) AS total_conversions\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n    INNER JOIN `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` AS t2 ON t1.audience_id = t2.audience_id\\n  GROUP BY\\n    t2.audience_segment\\n  ORDER BY\\n    total_conversions DESC\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"audience_segment\": \"Cart Abandoners\",\n      \"total_conversions\": 175430\n    },\n    {\n      \"audience_segment\": \"Geo-Targeted Shoppers\",\n      \"total_conversions\": 148821\n    },\n    {\n      \"audience_segment\": \"Loyalty Program Members\",\n      \"total_conversions\": 145905\n    },\n    {\n      \"audience_segment\": \"Frequent Buyers\",\n      \"total_conversions\": 142301\n    },\n    {\n      \"audience_segment\": \"Deal Hunters\",\n      \"total_conversions\": 141497\n    },\n    {\n      \"audience_segment\": \"Lookalike Audiences\",\n      \"total_conversions\": 137501\n    },\n    {\n      \"audience_segment\": \"New to Category\",\n      \"total_conversions\": 130697\n    },\n    {\n      \"audience_segment\": \"Promo Responders\",\n      \"total_conversions\": 122216\n    },\n    {\n      \"audience_segment\": \"Seasonal Shoppers\",\n      \"total_conversions\": 112235\n    },\n    {\n      \"audience_segment\": \"App Engaged Shoppers\",\n      \"total_conversions\": 106473\n    },\n    {\n      \"audience_segment\": \"New to Brand\",\n      \"total_conversions\": 94798\n    },\n    {\n      \"audience_segment\": \"High-Intent Visitors\",\n      \"total_conversions\": 93765\n    },\n    {\n      \"audience_segment\": \"Frequent Browsers\",\n      \"total_conversions\": 85921\n    },\n    {\n      \"audience_segment\": \"Brand Interactors\",\n      \"total_conversions\": 72356\n    },\n    {\n      \"audience_segment\": \"Category Enthusiasts\",\n      \"total_conversions\": 72173\n    },\n    {\n      \"audience_segment\": \"Auto-Replenish Candidates\",\n      \"total_conversions\": 47004\n    },\n    {\n      \"audience_segment\": \"Brand Loyalists\",\n      \"total_conversions\": 43964\n    },\n    {\n      \"audience_segment\": \"Value Shoppers\",\n      \"total_conversions\": 39209\n    },\n    {\n      \"audience_segment\": \"Churn Risk\",\n      \"total_conversions\": 38452\n    },\n    {\n      \"audience_segment\": \"Repeat Buyers\",\n      \"total_conversions\": 34849\n  }],\n  \"nl_results\": \"The total conversions by audience segment are:\\n- Cart Abandoners: 175,430\\n- Geo-Targeted Shoppers: 148,821\\n- Loyalty Program Members: 145,905\\n- Frequent Buyers: 142,301\\n- Deal Hunters: 141,497\\n- Lookalike Audiences: 137,501\\n- New to Category: 130,697\\n- Promo Responders: 122,216\\n- Seasonal Shoppers: 112,235\\n- App Engaged Shoppers: 106,473\\n- New to Brand: 94,798\\n- High-Intent Visitors: 93,765\\n- Frequent Browsers: 85,921\\n- Brand Interactors: 72,356\\n- Category Enthusiasts: 72,173\\n- Auto-Replenish Candidates: 47,004\\n- Brand Loyalists: 43,964\\n- Value Shoppers: 39,209\\n- Churn Risk: 38,452\\n- Repeat Buyers: 34,849\"\n}\n```"}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "8e17tlVe", "timestamp": 1757660161.306614}, {"content": {"parts": [{"functionCall": {"id": "adk-88b8aab4-3e36-4b5f-9701-6326592fad3b", "args": {"question": "Pie chart of conversions by audience segment."}, "name": "call_viz_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7596}], "cachedContentTokenCount": 7596, "candidatesTokenCount": 14, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 14}], "promptTokenCount": 9462, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 9462}], "thoughtsTokenCount": 106, "totalTokenCount": 9582, "trafficType": "ON_DEMAND"}, "invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "IWQM1gda", "timestamp": 1757660161.307592}, {"content": {"parts": [{"functionResponse": {"id": "adk-88b8aab4-3e36-4b5f-9701-6326592fad3b", "name": "call_viz_agent", "response": {"text": "I've created a pie chart showing 'Conversions by Audience Segment'. Each slice represents an audience segment, and its size corresponds to the 'total_conversions' for that segment. This chart effectively illustrates the proportion of conversions contributed by different audience segments.\n\nLet me know if you'd like to explore other aspects of this data or create different visualizations!", "images": []}}}], "role": "user"}, "invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {"chart_type": "pie", "x_axis_label": "", "y_axis_label": "", "x": [], "y": [], "categories": ["Cart Abandoners", "Geo-Targeted Shoppers", "Loyalty Program Members", "Frequent Buyers", "Deal Hunters", "Lookalike Audiences", "New to Category", "Promo Responders", "Seasonal Shoppers", "App Engaged Shoppers", "New to Brand", "High-Intent Visitors", "Frequent Browsers", "Brand Interactors", "Category Enthusiasts", "Auto-Replenish Candidates", "Brand Loyalists", "Value Shoppers", "Churn Risk", "Repeat Buyers"], "values": [175430, 148821, 145905, 142301, 141497, 137501, 130697, 122216, 112235, 106473, 94798, 93765, 85921, 72356, 72173, 47004, 43964, 39209, 38452, 34849], "title": "Conversions by Audience Segment", "stages": [], "subcategories": [], "dv_agent_output": "I've created a pie chart showing 'Conversions by Audience Segment'. Each slice represents an audience segment, and its size corresponds to the 'total_conversions' for that segment. This chart effectively illustrates the proportion of conversions contributed by different audience segments.\n\nLet me know if you'd like to explore other aspects of this data or create different visualizations!"}, "artifactDelta": {"chart_20250912_122618.png": 0}, "requestedAuthConfigs": {}}, "id": "udIeRYVj", "timestamp": 1757660188.379288}, {"content": {"parts": [{"text": "**Result:**\nThe total conversions by audience segment are:\n- Cart Abandoners: 175,430\n- Geo-Targeted Shoppers: 148,821\n- Loyalty Program Members: 145,905\n- Frequent Buyers: 142,301\n- Deal Hunters: 141,497\n- Lookalike Audiences: 137,501\n- New to Category: 130,697\n- Promo Responders: 122,216\n- Seasonal Shoppers: 112,235\n- App Engaged Shoppers: 106,473\n- New to Brand: 94,798\n- High-Intent Visitors: 93,765\n- Frequent Browsers: 85,921\n- Brand Interactors: 72,356\n- Category Enthusiasts: 72,173\n- Auto-Replenish Candidates: 47,004\n- Brand Loyalists: 43,964\n- Value Shoppers: 39,209\n- Churn Risk: 38,452\n- Repeat Buyers: 34,849\n\nA pie chart showing 'Conversions by Audience Segment' has been created. Each slice represents an audience segment, and its size corresponds to the 'total_conversions' for that segment. This chart effectively illustrates the proportion of conversions contributed by different audience segments."}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7576}], "cachedContentTokenCount": 7576, "candidatesTokenCount": 338, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 338}], "promptTokenCount": 9629, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 9629}], "thoughtsTokenCount": 148, "totalTokenCount": 10115, "trafficType": "ON_DEMAND"}, "invocationId": "e-3c0f58c9-4384-4002-a6bb-1fb09377f4ee", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "MQkEQ2UL", "timestamp": 1757660188.380286}]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:55:21.234070Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:56:38.920968Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1:17.687</t>
         </is>
       </c>
     </row>
@@ -589,23 +686,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Result: The chart above displays the daily reach for July 2025. This area chart effectively visualizes the trend of daily reach over the month. We can observe a general decline in daily reach from the beginning to the end of July, with a notable increase in reach towards the very end of the month.</t>
+          <t>Result: The area chart visualizes the daily reach for July 2025. It shows a general downward trend in daily reach throughout the month, with a significant increase at the very end of July.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>SELECT
-    PARSE_DATE('%Y-%m-%d', FORMAT_DATE('%Y-%m-%d', t1.date)) AS daily_date,
+    t1.date,
     SUM(t1.reach) AS total_daily_reach
   FROM
     `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1
   WHERE
-    t1.date &gt;= '2025-07-01'
-    AND t1.date &lt; '2025-08-01'
+    t1.date BETWEEN '2025-07-01' AND '2025-07-31'
   GROUP BY
-    daily_date
+    t1.date
   ORDER BY
-    daily_date
+    t1.date
   LIMIT 500</t>
         </is>
       </c>
@@ -615,19 +711,34 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.9256</v>
+        <v>0.9036</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9059</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>[{"invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {"all_db_settings": {"use_database": "BigQuery"}, "database_settings": {"bq_project_id": "acn-cda", "bq_dataset_id": "RMN_Campaign_Dataset_Dev", "bq_ddl_schema": "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", "transpile_to_bigquery": true, "process_input_errors": true, "process_tool_output_errors": true, "number_of_candidates": 1, "model": "gemini-2.5-flash", "temperature": 0.01, "generate_sql_type": "dc"}}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "IqteIHou", "timestamp": 1757481629.437732}, {"content": {"parts": [{"functionCall": {"id": "adk-77e814f7-009a-42b2-87fb-9cae002aece0", "args": {"question": "daily reach for July 2025"}, "name": "call_db_agent"}}], "role": "model"}, "usageMetadata": {"candidatesTokenCount": 15, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 15}], "promptTokenCount": 8269, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8269}], "thoughtsTokenCount": 352, "totalTokenCount": 8636, "trafficType": "ON_DEMAND"}, "invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "BRu23PP3", "timestamp": 1757481629.439582}, {"content": {"parts": [{"functionResponse": {"id": "adk-77e814f7-009a-42b2-87fb-9cae002aece0", "name": "call_db_agent", "response": {"result": "```json\n{\n  \"explain\": \"The SQL query calculates the daily reach for July 2025. It selects the date and sums the `reach` column from the `campaign_performance` table. It filters the data for dates between '2025-07-01' and '2025-07-31' (exclusive of '2025-08-01'). The results are grouped by date and ordered by date.\",\n  \"sql\": \"SELECT\\n    PARSE_DATE('%Y-%m-%d', FORMAT_DATE('%Y-%m-%d', t1.date)) AS daily_date,\\n    SUM(t1.reach) AS total_daily_reach\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  WHERE\\n    t1.date &gt;= '2025-07-01'\\n    AND t1.date &lt; '2025-08-01'\\n  GROUP BY\\n    daily_date\\n  ORDER BY\\n    daily_date\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"daily_date\": \"2025-07-01\",\n      \"total_daily_reach\": 5995346\n    },\n    {\n      \"daily_date\": \"2025-07-02\",\n      \"total_daily_reach\": 6031607\n    },\n    {\n      \"daily_date\": \"2025-07-03\",\n      \"total_daily_reach\": 5917203\n    },\n    {\n      \"daily_date\": \"2025-07-04\",\n      \"total_daily_reach\": 5791901\n    },\n    {\n      \"daily_date\": \"2025-07-05\",\n      \"total_daily_reach\": 5624287\n    },\n    {\n      \"daily_date\": \"2025-07-06\",\n      \"total_daily_reach\": 5629257\n    },\n    {\n      \"daily_date\": \"2025-07-07\",\n      \"total_daily_reach\": 5485384\n    },\n    {\n      \"daily_date\": \"2025-07-08\",\n      \"total_daily_reach\": 5326269\n    },\n    {\n      \"daily_date\": \"2025-07-09\",\n      \"total_daily_reach\": 5230622\n    },\n    {\n      \"daily_date\": \"2025-07-10\",\n      \"total_daily_reach\": 5086002\n    },\n    {\n      \"daily_date\": \"2025-07-11\",\n      \"total_daily_reach\": 4941544\n    },\n    {\n      \"daily_date\": \"2025-07-12\",\n      \"total_daily_reach\": 4788686\n    },\n    {\n      \"daily_date\": \"2025-07-13\",\n      \"total_daily_reach\": 4588218\n    },\n    {\n      \"daily_date\": \"2025-07-14\",\n      \"total_daily_reach\": 4374487\n    },\n    {\n      \"daily_date\": \"2025-07-15\",\n      \"total_daily_reach\": 4287538\n    },\n    {\n      \"daily_date\": \"2025-07-16\",\n      \"total_daily_reach\": 4094771\n    },\n    {\n      \"daily_date\": \"2025-07-17\",\n      \"total_daily_reach\": 4007549\n    },\n    {\n      \"daily_date\": \"2025-07-18\",\n      \"total_daily_reach\": 3767491\n    },\n    {\n      \"daily_date\": \"2025-07-19\",\n      \"total_daily_reach\": 3586414\n    },\n    {\n      \"daily_date\": \"2025-07-20\",\n      \"total_daily_reach\": 3487322\n    },\n    {\n      \"daily_date\": \"2025-07-21\",\n      \"total_daily_reach\": 3237921\n    },\n    {\n      \"daily_date\": \"2025-07-22\",\n      \"total_daily_reach\": 3035686\n    },\n    {\n      \"daily_date\": \"2025-07-23\",\n      \"total_daily_reach\": 2858238\n    },\n    {\n      \"daily_date\": \"2025-07-24\",\n      \"total_daily_reach\": 2634915\n    },\n    {\n      \"daily_date\": \"2025-07-25\",\n      \"total_daily_reach\": 2456400\n    },\n    {\n      \"daily_date\": \"2025-07-26\",\n      \"total_daily_reach\": 2370349\n    },\n    {\n      \"daily_date\": \"2025-07-27\",\n      \"total_daily_reach\": 2094288\n    },\n    {\n      \"daily_date\": \"2025-07-28\",\n      \"total_daily_reach\": 1911266\n    },\n    {\n      \"daily_date\": \"2025-07-29\",\n      \"total_daily_reach\": 3813140\n    },\n    {\n      \"daily_date\": \"2025-07-30\",\n      \"total_daily_reach\": 5533606\n    },\n    {\n      \"daily_date\": \"2025-07-31\",\n      \"total_daily_reach\": 7640471\n    }\n  ],\n  \"nl_results\": \"Here is the daily reach for July 2025:\\nJuly 1, 2025: 5,995,346\\nJuly 2, 2025: 6,031,607\\nJuly 3, 2025: 5,917,203\\nJuly 4, 2025: 5,791,901\\nJuly 5, 2025: 5,624,287\\nJuly 6, 2025: 5,629,257\\nJuly 7, 2025: 5,485,384\\nJuly 8, 2025: 5,326,269\\nJuly 9, 2025: 5,230,622\\nJuly 10, 2025: 5,086,002\\nJuly 11, 2025: 4,941,544\\nJuly 12, 2025: 4,788,686\\nJuly 13, 2025: 4,588,218\\nJuly 14, 2025: 4,374,487\\nJuly 15, 2025: 4,287,538\\nJuly 16, 2025: 4,094,771\\nJuly 17, 2025: 4,007,549\\nJuly 18, 2025: 3,767,491\\nJuly 19, 2025: 3,586,414\\nJuly 20, 2025: 3,487,322\\nJuly 21, 2025: 3,237,921\\nJuly 22, 2025: 3,035,686\\nJuly 23, 2025: 2,858,238\\nJuly 24, 2025: 2,634,915\\nJuly 25, 2025: 2,456,400\\nJuly 26, 2025: 2,370,349\\nJuly 27, 2025: 2,094,288\\nJuly 28, 2025: 1,911,266\\nJuly 29, 2025: 3,813,140\\nJuly 30, 2025: 5,533,606\\nJuly 31, 2025: 7,640,471\"\n}\n```"}}}], "role": "user"}, "invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {"sql_query": "SELECT\n    PARSE_DATE('%Y-%m-%d', FORMAT_DATE('%Y-%m-%d', t1.date)) AS daily_date,\n    SUM(t1.reach) AS total_daily_reach\n  FROM\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\n  WHERE\n    t1.date &gt;= '2025-07-01'\n    AND t1.date &lt; '2025-08-01'\n  GROUP BY\n    daily_date\n  ORDER BY\n    daily_date\n  LIMIT 500", "query_result": [{"daily_date": "2025-07-01", "total_daily_reach": 5995346.0}, {"daily_date": "2025-07-02", "total_daily_reach": 6031607.0}, {"daily_date": "2025-07-03", "total_daily_reach": 5917203.0}, {"daily_date": "2025-07-04", "total_daily_reach": 5791901.0}, {"daily_date": "2025-07-05", "total_daily_reach": 5624287.0}, {"daily_date": "2025-07-06", "total_daily_reach": 5629257.0}, {"daily_date": "2025-07-07", "total_daily_reach": 5485384.0}, {"daily_date": "2025-07-08", "total_daily_reach": 5326269.0}, {"daily_date": "2025-07-09", "total_daily_reach": 5230622.0}, {"daily_date": "2025-07-10", "total_daily_reach": 5086002.0}, {"daily_date": "2025-07-11", "total_daily_reach": 4941544.0}, {"daily_date": "2025-07-12", "total_daily_reach": 4788686.0}, {"daily_date": "2025-07-13", "total_daily_reach": 4588218.0}, {"daily_date": "2025-07-14", "total_daily_reach": 4374487.0}, {"daily_date": "2025-07-15", "total_daily_reach": 4287538.0}, {"daily_date": "2025-07-16", "total_daily_reach": 4094771.0}, {"daily_date": "2025-07-17", "total_daily_reach": 4007549.0}, {"daily_date": "2025-07-18", "total_daily_reach": 3767491.0}, {"daily_date": "2025-07-19", "total_daily_reach": 3586414.0}, {"daily_date": "2025-07-20", "total_daily_reach": 3487322.0}, {"daily_date": "2025-07-21", "total_daily_reach": 3237921.0}, {"daily_date": "2025-07-22", "total_daily_reach": 3035686.0}, {"daily_date": "2025-07-23", "total_daily_reach": 2858238.0}, {"daily_date": "2025-07-24", "total_daily_reach": 2634915.0}, {"daily_date": "2025-07-25", "total_daily_reach": 2456400.0}, {"daily_date": "2025-07-26", "total_daily_reach": 2370349.0}, {"daily_date": "2025-07-27", "total_daily_reach": 2094288.0}, {"daily_date": "2025-07-28", "total_daily_reach": 1911266.0}, {"daily_date": "2025-07-29", "total_daily_reach": 3813140.0}, {"daily_date": "2025-07-30", "total_daily_reach": 5533606.0}, {"daily_date": "2025-07-31", "total_daily_reach": 7640471.0}], "db_agent_output": "```json\n{\n  \"explain\": \"The SQL query calculates the daily reach for July 2025. It selects the date and sums the `reach` column from the `campaign_performance` table. It filters the data for dates between '2025-07-01' and '2025-07-31' (exclusive of '2025-08-01'). The results are grouped by date and ordered by date.\",\n  \"sql\": \"SELECT\\n    PARSE_DATE('%Y-%m-%d', FORMAT_DATE('%Y-%m-%d', t1.date)) AS daily_date,\\n    SUM(t1.reach) AS total_daily_reach\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  WHERE\\n    t1.date &gt;= '2025-07-01'\\n    AND t1.date &lt; '2025-08-01'\\n  GROUP BY\\n    daily_date\\n  ORDER BY\\n    daily_date\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"daily_date\": \"2025-07-01\",\n      \"total_daily_reach\": 5995346\n    },\n    {\n      \"daily_date\": \"2025-07-02\",\n      \"total_daily_reach\": 6031607\n    },\n    {\n      \"daily_date\": \"2025-07-03\",\n      \"total_daily_reach\": 5917203\n    },\n    {\n      \"daily_date\": \"2025-07-04\",\n      \"total_daily_reach\": 5791901\n    },\n    {\n      \"daily_date\": \"2025-07-05\",\n      \"total_daily_reach\": 5624287\n    },\n    {\n      \"daily_date\": \"2025-07-06\",\n      \"total_daily_reach\": 5629257\n    },\n    {\n      \"daily_date\": \"2025-07-07\",\n      \"total_daily_reach\": 5485384\n    },\n    {\n      \"daily_date\": \"2025-07-08\",\n      \"total_daily_reach\": 5326269\n    },\n    {\n      \"daily_date\": \"2025-07-09\",\n      \"total_daily_reach\": 5230622\n    },\n    {\n      \"daily_date\": \"2025-07-10\",\n      \"total_daily_reach\": 5086002\n    },\n    {\n      \"daily_date\": \"2025-07-11\",\n      \"total_daily_reach\": 4941544\n    },\n    {\n      \"daily_date\": \"2025-07-12\",\n      \"total_daily_reach\": 4788686\n    },\n    {\n      \"daily_date\": \"2025-07-13\",\n      \"total_daily_reach\": 4588218\n    },\n    {\n      \"daily_date\": \"2025-07-14\",\n      \"total_daily_reach\": 4374487\n    },\n    {\n      \"daily_date\": \"2025-07-15\",\n      \"total_daily_reach\": 4287538\n    },\n    {\n      \"daily_date\": \"2025-07-16\",\n      \"total_daily_reach\": 4094771\n    },\n    {\n      \"daily_date\": \"2025-07-17\",\n      \"total_daily_reach\": 4007549\n    },\n    {\n      \"daily_date\": \"2025-07-18\",\n      \"total_daily_reach\": 3767491\n    },\n    {\n      \"daily_date\": \"2025-07-19\",\n      \"total_daily_reach\": 3586414\n    },\n    {\n      \"daily_date\": \"2025-07-20\",\n      \"total_daily_reach\": 3487322\n    },\n    {\n      \"daily_date\": \"2025-07-21\",\n      \"total_daily_reach\": 3237921\n    },\n    {\n      \"daily_date\": \"2025-07-22\",\n      \"total_daily_reach\": 3035686\n    },\n    {\n      \"daily_date\": \"2025-07-23\",\n      \"total_daily_reach\": 2858238\n    },\n    {\n      \"daily_date\": \"2025-07-24\",\n      \"total_daily_reach\": 2634915\n    },\n    {\n      \"daily_date\": \"2025-07-25\",\n      \"total_daily_reach\": 2456400\n    },\n    {\n      \"daily_date\": \"2025-07-26\",\n      \"total_daily_reach\": 2370349\n    },\n    {\n      \"daily_date\": \"2025-07-27\",\n      \"total_daily_reach\": 2094288\n    },\n    {\n      \"daily_date\": \"2025-07-28\",\n      \"total_daily_reach\": 1911266\n    },\n    {\n      \"daily_date\": \"2025-07-29\",\n      \"total_daily_reach\": 3813140\n    },\n    {\n      \"daily_date\": \"2025-07-30\",\n      \"total_daily_reach\": 5533606\n    },\n    {\n      \"daily_date\": \"2025-07-31\",\n      \"total_daily_reach\": 7640471\n    }\n  ],\n  \"nl_results\": \"Here is the daily reach for July 2025:\\nJuly 1, 2025: 5,995,346\\nJuly 2, 2025: 6,031,607\\nJuly 3, 2025: 5,917,203\\nJuly 4, 2025: 5,791,901\\nJuly 5, 2025: 5,624,287\\nJuly 6, 2025: 5,629,257\\nJuly 7, 2025: 5,485,384\\nJuly 8, 2025: 5,326,269\\nJuly 9, 2025: 5,230,622\\nJuly 10, 2025: 5,086,002\\nJuly 11, 2025: 4,941,544\\nJuly 12, 2025: 4,788,686\\nJuly 13, 2025: 4,588,218\\nJuly 14, 2025: 4,374,487\\nJuly 15, 2025: 4,287,538\\nJuly 16, 2025: 4,094,771\\nJuly 17, 2025: 4,007,549\\nJuly 18, 2025: 3,767,491\\nJuly 19, 2025: 3,586,414\\nJuly 20, 2025: 3,487,322\\nJuly 21, 2025: 3,237,921\\nJuly 22, 2025: 3,035,686\\nJuly 23, 2025: 2,858,238\\nJuly 24, 2025: 2,634,915\\nJuly 25, 2025: 2,456,400\\nJuly 26, 2025: 2,370,349\\nJuly 27, 2025: 2,094,288\\nJuly 28, 2025: 1,911,266\\nJuly 29, 2025: 3,813,140\\nJuly 30, 2025: 5,533,606\\nJuly 31, 2025: 7,640,471\"\n}\n```"}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "dK6KfEje", "timestamp": 1757481700.493294}, {"content": {"parts": [{"functionCall": {"id": "adk-6bd34d20-e4bb-4216-b99a-3b6980cc55b3", "args": {"question": "Area chart of daily reach for July 2025."}, "name": "call_viz_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7658}], "cachedContentTokenCount": 7658, "candidatesTokenCount": 19, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 19}], "promptTokenCount": 10593, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 10593}], "thoughtsTokenCount": 119, "totalTokenCount": 10731, "trafficType": "ON_DEMAND"}, "invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "TUd9tDgI", "timestamp": 1757481700.495342}, {"content": {"parts": [{"functionResponse": {"id": "adk-6bd34d20-e4bb-4216-b99a-3b6980cc55b3", "name": "call_viz_agent", "response": {"text": "The chart above displays the daily reach for July 2025. This area chart effectively visualizes the trend of daily reach over the month. We can observe a general decline in daily reach from the beginning to the end of July, with a notable increase in reach towards the very end of the month.", "images": []}}}], "role": "user"}, "invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {"chart_type": "area", "x_axis_label": "Date", "y_axis_label": "Total Daily Reach", "x": [], "y": [], "categories": ["2025-07-01", "2025-07-02", "2025-07-03", "2025-07-04", "2025-07-05", "2025-07-06", "2025-07-07", "2025-07-08", "2025-07-09", "2025-07-10", "2025-07-11", "2025-07-12", "2025-07-13", "2025-07-14", "2025-07-15", "2025-07-16", "2025-07-17", "2025-07-18", "2025-07-19", "2025-07-20", "2025-07-21", "2025-07-22", "2025-07-23", "2025-07-24", "2025-07-25", "2025-07-26", "2025-07-27", "2025-07-28", "2025-07-29", "2025-07-30", "2025-07-31"], "values": [5995346, 6031607, 5917203, 5791901, 5624287, 5629257, 5485384, 5326269, 5230622, 5086002, 4941544, 4788686, 4588218, 4374487, 4287538, 4094771, 4007549, 3767491, 3586414, 3487322, 3237921, 3035686, 2858238, 2634915, 2456400, 2370349, 2094288, 1911266, 3813140, 5533606, 7640471], "title": "Daily Reach for July 2025", "stages": [], "subcategories": [], "dv_agent_output": "The chart above displays the daily reach for July 2025. This area chart effectively visualizes the trend of daily reach over the month. We can observe a general decline in daily reach from the beginning to the end of July, with a notable increase in reach towards the very end of the month."}, "artifactDelta": {"chart_20250910_105209.png": 0}, "requestedAuthConfigs": {}}, "id": "aV7zhWZM", "timestamp": 1757481742.740417}, {"content": {"parts": [{"text": "Result: The chart above displays the daily reach for July 2025. This area chart effectively visualizes the trend of daily reach over the month. We can observe a general decline in daily reach from the beginning to the end of July, with a notable increase in reach towards the very end of the month."}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7642}], "cachedContentTokenCount": 7642, "candidatesTokenCount": 64, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 64}], "promptTokenCount": 10756, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 10756}], "thoughtsTokenCount": 119, "totalTokenCount": 10939, "trafficType": "ON_DEMAND"}, "invocationId": "e-40d05628-6d99-4926-b6d2-3fb9ef9d6992", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "OhR2Sxb0", "timestamp": 1757481742.741647}]</t>
+          <t>[{"invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"all_db_settings": {"use_database": "BigQuery"}, "database_settings": {"bq_project_id": "acn-cda", "bq_dataset_id": "RMN_Campaign_Dataset_Dev", "bq_ddl_schema": "CREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` (\n  `audience_id` STRING,\n  `audience_segment` STRING,\n  `audience_desc` STRING,\n  `platform_audience_id` STRING,\n  `is_converted` INTEGER,\n  `conversion_value` FLOAT,\n  `audience_size` INTEGER,\n  `audience_source` STRING,\n  `audience_platform` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.audience_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0012','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00029',1,631392.0,4328,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0073','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00113',1,976836.0,3789,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0018','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00124',1,40203.0,1993,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0088','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00170',1,223193.0,4264,'2P','Meta');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.audience_data` VALUES\n('CONS_0017','App Engaged Shoppers','\u2265 3 sessions in retailer app over past month','MET_AUD_00234',1,686242.0,3137,'2P','Meta');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` (\n  `advertiser_id` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_grp_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATE,\n  `end_date` DATE,\n  `budget` FLOAT,\n  `planned_spend` FLOAT,\n  `strategy_description` STRING,\n  `status` STRING,\n  `channel_id` STRING,\n  `creative_id` STRING,\n  `strategy_category` STRING,\n  `strategy_id` STRING,\n  `site_id` STRING,\n  `campaign_name` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000001','D04_C04_B03_S002_Var459','BRAND_003','Ben &amp; Jerry's','Sponsored Product','Onsite','Consideration','App Installs',2025-08-21,2025-10-24,13184.67,407.28,'Retailer Recommended Strategy','Planned','CH_ONS15','CR_001','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_001','CMP_2025_0001 - Ben &amp; Jerry's - Onsite - Consideration - Sponsored Product - 20250821-20251024');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_01','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite','Consideration','App Installs',2025-05-14,2025-06-02,13184.67,1619.37,'CPA-Optimized','Completed','CH_ONS15','CR_002','Optimization-Based','Strategy-005','SITE_002','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000003','D01_C01_B02_S002_Var412','BRAND_038','Sunsilk','Sponsored Product','Onsite','Consideration','App Installs',2025-08-03,2025-08-22,13184.67,1204.75,'Budget Pacing','Active','CH_ONS15','CR_003','Optimization-Based','Strategy-004','SITE_003','CMP_2025_0001 - Sunsilk - Onsite - Consideration - Sponsored Product - 20250803-20250822');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_02','AD_00000004','D04_C04_B01_S001','BRAND_022','Magnum','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-12,13184.67,2578.34,'Retailer Recommended Strategy','Active','CH_ONS15','CR_004','AI/ML-Driven or Custom Strategies','Strategy-026','SITE_004','CMP_2025_0001 - Magnum - Onsite - Consideration - Sponsored Product - 20250802-20250812');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_metadata` VALUES\n('ADV_2025_B','CMP_2025_0001','CMP_2025_0001_ADGRP_03','AD_00000005','D01_C01_B03_S003','BRAND_040','TRESemme','Sponsored Product','Onsite','Consideration','App Installs',2025-08-02,2025-08-18,13184.67,709.28,'Long-Tail Keywords','Active','CH_ONS15','CR_005','Keyword-Level','Strategy-018','SITE_005','CMP_2025_0001 - TRESemme - Onsite - Consideration - Sponsored Product - 20250802-20250818');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` (\n  `campaign_id` STRING,\n  `campaign_name` STRING,\n  `campaign_ad_id` STRING,\n  `product_ids` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `total_campaign_budget` FLOAT,\n  `planned_spend` FLOAT,\n  `objective` STRING,\n  `sub_objective` STRING,\n  `start_date` DATETIME,\n  `end_date` DATETIME,\n  `status` STRING,\n  `date` DATETIME,\n  `daily_spend` FLOAT,\n  `actual_spend_to_date` FLOAT,\n  `impressions` FLOAT,\n  `frequency` FLOAT,\n  `reach` FLOAT,\n  `clicks` FLOAT,\n  `ctr_percent` FLOAT,\n  `conversions` FLOAT,\n  `conversion_rate_percent` FLOAT,\n  `attributed_sales_value` FLOAT,\n  `roas` FLOAT,\n  `cpc` FLOAT,\n  `cpa` FLOAT,\n  `remaining_budget` FLOAT,\n  `video_starts` INTEGER,\n  `video_plays` INTEGER,\n  `video_first_quartile` INTEGER,\n  `video_midpoint` INTEGER,\n  `video_third_quartile` INTEGER,\n  `video_completions` INTEGER,\n  `video_completion_rate_percent` FLOAT,\n  `avg_watch_time` FLOAT,\n  `add_to_cart_events` INTEGER,\n  `new_to_brand_conversions` INTEGER,\n  `dwell_time` INTEGER,\n  `gross_rating_point` FLOAT,\n  `target_audience_rating_point` FLOAT,\n  `delivered_messages` FLOAT,\n  `message_opens` FLOAT,\n  `unsubscribe_bounce_rates` FLOAT,\n  `extraction_date` STRING,\n  `audience_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-14 00:00:00,80.96849999999999,80.96849999999999,2824.0,2.05,1377.0,105.0,2.5,11.0,10.48,843.69,10.42,0.77,7.36,1538.4015,0,0,0,0,0,0,0.0,0.0,123,5,10,nan,nan,nan,nan,nan,'2025-08-19','CONS_0013');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-15 00:00:00,80.96849999999999,161.93699999999998,9935.0,2.17,4578.0,88.0,0.9,15.0,15.0,591.88,7.31,0.92,5.4,1457.433,0,0,0,0,0,0,0.0,0.0,949,4,19,nan,nan,nan,nan,nan,'2025-08-19','CONS_0087');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-16 00:00:00,80.96849999999999,242.90549999999996,9279.0,3.2,2899.0,76.0,0.9,7.0,9.21,826.69,10.21,1.07,11.57,1376.4645,0,0,0,0,0,0,0.0,0.0,704,4,12,nan,nan,nan,nan,nan,'2025-08-19','CONS_0048');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-17 00:00:00,80.96849999999999,323.87399999999997,7873.0,2.44,3226.0,74.0,0.94,6.0,8.11,489.05,6.04,1.09,13.49,1295.4959999999999,0,0,0,0,0,0,0.0,0.0,503,2,27,nan,nan,nan,nan,nan,'2025-08-19','CONS_0049');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` VALUES\n('CMP_2025_0001','CMP_2025_0001 - Liquid I.V. - Onsite - Consideration - Sponsored Product - 20250514-20250602','AD_00000002','D01_C03_B01_S002','BRAND_020','Liquid I.V.','Sponsored Product','Onsite',13184.67,1619.37,'Consideration','App Installs',2025-05-14 00:00:00,2025-06-02 00:00:00,'Completed',2025-05-18 00:00:00,80.96849999999999,404.8425,3615.0,3.4,1063.0,96.0,2.5,12.0,12.5,950.57,11.74,0.84,6.75,1214.5275,0,0,0,0,0,0,0.0,0.0,87,6,45,nan,nan,nan,nan,nan,'2025-08-19','CONS_0083');\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` (\n  `campaign_name` STRING,\n  `session_id` STRING,\n  `campaign_ad_id` STRING,\n  `product_id` STRING,\n  `event_time` DATETIME,\n  `event_type` STRING,\n  `event_id` INTEGER,\n  `user_id` STRING,\n  `page_url` STRING,\n  `referrer_url` STRING,\n  `media_type` STRING,\n  `channels` STRING,\n  `device_type` STRING,\n  `traffic_source` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `avg_time_on_site_sec` FLOAT,\n  `order_id` INTEGER,\n  `status` STRING,\n  `page_view` INTEGER,\n  `add_to_cart` INTEGER,\n  `purchase` INTEGER\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:09:00,'Page_View',1,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:14:00,'Add_to_Cart',2,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,&lt;NA&gt;,'Active',0,1,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2534 - Dove - Channel-CTV - Awareness - CTV - 20250804-20250831','S_025333','AD_00025333','D01_C01_B01_S001',2025-08-17 03:16:00,'Purchase',3,'USER_6TQY9W','https://www.target.com/dove','NA','ctv','channel-ctv','tablet','Organic','BRAND_013','Dove',570.16,1001210,'Active',0,0,1);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2620 - Dove - Channel-CTV - Consideration - CTV - 20250802-20250909','S_026192','AD_00026192','D01_C01_B01_S001',2025-08-30 08:30:00,'Page_View',1,'USER_9MQYYT','https://www.costco.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',125.76,&lt;NA&gt;,'Active',1,0,0);\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.clickstream_data` VALUES\n('CMP_2025_2595 - Dove - Channel-CTV - Consideration - CTV - 20250501-20250529','S_025945','AD_00025945','D01_C01_B01_S001',2025-05-28 07:23:00,'Page_View',1,'USER_I47QNE','https://www.target.com/dove','NA','ctv','channel-ctv','mobile','Organic','BRAND_013','Dove',285.12,&lt;NA&gt;,'Completed',1,0,0);\n\nCREATE OR REPLACE TABLE `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` (\n  `order_id` INTEGER,\n  `transaction_date` DATETIME,\n  `user_id` STRING,\n  `sku_id` STRING,\n  `order_amount` INTEGER,\n  `currency` STRING,\n  `unit_sold` INTEGER,\n  `department_code` STRING,\n  `category_code` STRING,\n  `brand_id` STRING,\n  `brand_name` STRING,\n  `sku_desc` STRING,\n  `department_desc` STRING,\n  `category_desc` STRING,\n  `vendor_id` STRING,\n  `vendor_name` STRING,\n  `campaign_id` STRING,\n  `campaign_ad_id` STRING,\n  `advertiser_id` STRING\n);\n\n-- Example values for table `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data`:\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S001',459,'USD',18,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S003',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000000,2025-05-09 15:23:42,'USER_JTS5R0','D01_C01_B01_S002',47,'USD',2,'D01','D01_C01','D01_C01_B01','Dove','Dove Deep Moisture Body Wash 500ml','Beauty &amp; Wellbeing','Hair Care','VEND008','Vendor 8','CMP_2025_5270','AD_00006434','ADV_2025_B');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S001',29,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Intense Repair Shampoo 350ml','Beauty &amp; Wellbeing','Hair Care','VEND001','Vendor 1','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\nINSERT INTO `acn-cda.RMN_Campaign_Dataset_Dev.transaction_data` VALUES\n(1000001,2025-08-14 16:39:31,'USER_U67NM7','D01_C01_B01_S003',17,'USD',1,'D01','D01_C01','D01_C01_B01','Dove','Dove Original Antiperspirant Roll-On 50ml','Beauty &amp; Wellbeing','Hair Care','VEND006','Vendor 6','CMP_2025_2901','AD_00016384','ADV_2025_D');\n\n", "transpile_to_bigquery": true, "process_input_errors": true, "process_tool_output_errors": true, "number_of_candidates": 1, "model": "gemini-2.5-flash", "temperature": 0.01, "generate_sql_type": "dc"}}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "CNswMqZs", "timestamp": 1757660199.094295}, {"content": {"parts": [{"functionCall": {"id": "adk-3b80196d-e0d0-44cb-a539-d73406320769", "args": {"question": "daily reach for July 2025 from campaign_performance table"}, "name": "call_db_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7610}], "cachedContentTokenCount": 7610, "candidatesTokenCount": 20, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 20}], "promptTokenCount": 8269, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 8269}], "thoughtsTokenCount": 245, "totalTokenCount": 8534, "trafficType": "ON_DEMAND"}, "invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "DFkMxcFF", "timestamp": 1757660199.095629}, {"content": {"parts": [{"functionResponse": {"id": "adk-3b80196d-e0d0-44cb-a539-d73406320769", "name": "call_db_agent", "response": {"result": "```json\n{\n  \"explain\": \"The SQL query retrieves the daily reach from the `campaign_performance` table for July 2025. It sums the `reach` for each day and filters the results to include only dates within July 2025. The results are then grouped and ordered by date.\",\n  \"sql\": \"SELECT\\n    t1.date,\\n    SUM(t1.reach) AS total_daily_reach\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  WHERE\\n    t1.date BETWEEN '2025-07-01' AND '2025-07-31'\\n  GROUP BY\\n    t1.date\\n  ORDER BY\\n    t1.date\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"date\": \"2025-07-01\",\n      \"total_daily_reach\": 5995346\n    },\n    {\n      \"date\": \"2025-07-02\",\n      \"total_daily_reach\": 6031607\n    },\n    {\n      \"date\": \"2025-07-03\",\n      \"total_daily_reach\": 5917203\n    },\n    {\n      \"date\": \"2025-07-04\",\n      \"total_daily_reach\": 5791901\n    },\n    {\n      \"date\": \"2025-07-05\",\n      \"total_daily_reach\": 5624287\n    },\n    {\n      \"date\": \"2025-07-06\",\n      \"total_daily_reach\": 5629257\n    },\n    {\n      \"date\": \"2025-07-07\",\n      \"total_daily_reach\": 5485384\n    },\n    {\n      \"date\": \"2025-07-08\",\n      \"total_daily_reach\": 5326269\n    },\n    {\n      \"date\": \"2025-07-09\",\n      \"total_daily_reach\": 5230622\n    },\n    {\n      \"date\": \"2025-07-10\",\n      \"total_daily_reach\": 5086002\n    },\n    {\n      \"date\": \"2025-07-11\",\n      \"total_daily_reach\": 4941544\n    },\n    {\n      \"date\": \"2025-07-12\",\n      \"total_daily_reach\": 4788686\n    },\n    {\n      \"date\": \"2025-07-13\",\n      \"total_daily_reach\": 4588218\n    },\n    {\n      \"date\": \"2025-07-14\",\n      \"total_daily_reach\": 4374487\n    },\n    {\n      \"date\": \"2025-07-15\",\n      \"total_daily_reach\": 4287538\n    },\n    {\n      \"date\": \"2025-07-16\",\n      \"total_daily_reach\": 4094771\n    },\n    {\n      \"date\": \"2025-07-17\",\n      \"total_daily_reach\": 4007549\n    },\n    {\n      \"date\": \"2025-07-18\",\n      \"total_daily_reach\": 3767491\n    },\n    {\n      \"date\": \"2025-07-19\",\n      \"total_daily_reach\": 3586414\n    },\n    {\n      \"date\": \"2025-07-20\",\n      \"total_daily_reach\": 3487322\n    },\n    {\n      \"date\": \"2025-07-21\",\n      \"total_daily_reach\": 3237921\n    },\n    {\n      \"date\": \"2025-07-22\",\n      \"total_daily_reach\": 3035686\n    },\n    {\n      \"date\": \"2025-07-23\",\n      \"total_daily_reach\": 2858238\n    },\n    {\n      \"date\": \"2025-07-24\",\n      \"total_daily_reach\": 2634915\n    },\n    {\n      \"date\": \"2025-07-25\",\n      \"total_daily_reach\": 2456400\n    },\n    {\n      \"date\": \"2025-07-26\",\n      \"total_daily_reach\": 2370349\n    },\n    {\n      \"date\": \"2025-07-27\",\n      \"total_daily_reach\": 2094288\n    },\n    {\n      \"date\": \"2025-07-28\",\n      \"total_daily_reach\": 1911266\n    },\n    {\n      \"date\": \"2025-07-29\",\n      \"total_daily_reach\": 3813140\n    },\n    {\n      \"date\": \"2025-07-30\",\n      \"total_daily_reach\": 5533606\n    },\n    {\n      \"date\": \"2025-07-31\",\n      \"total_daily_reach\": 7640471\n    }\n  ],\n  \"nl_results\": \"The daily reach for campaigns in July 2025 from the campaign performance table is as follows:\\nJuly 1: 5,995,346\\nJuly 2: 6,031,607\\nJuly 3: 5,917,203\\nJuly 4: 5,791,901\\nJuly 5: 5,624,287\\nJuly 6: 5,629,257\\nJuly 7: 5,485,384\\nJuly 8: 5,326,269\\nJuly 9: 5,230,622\\nJuly 10: 5,086,002\\nJuly 11: 4,941,544\\nJuly 12: 4,788,686\\nJuly 13: 4,588,218\\nJuly 14: 4,374,487\\nJuly 15: 4,287,538\\nJuly 16: 4,094,771\\nJuly 17: 4,007,549\\nJuly 18: 3,767,491\\nJuly 19: 3,586,414\\nJuly 20: 3,487,322\\nJuly 21: 3,237,921\\nJuly 22: 3,035,686\\nJuly 23: 2,858,238\\nJuly 24: 2,634,915\\nJuly 25: 2,456,400\\nJuly 26: 2,370,349\\nJuly 27: 2,094,288\\nJuly 28: 1,911,266\\nJuly 29: 3,813,140\\nJuly 30: 5,533,606\\nJuly 31: 7,640,471\"\n}\n```"}}}], "role": "user"}, "invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"sql_query": "SELECT\n    t1.date,\n    SUM(t1.reach) AS total_daily_reach\n  FROM\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\n  WHERE\n    t1.date BETWEEN '2025-07-01' AND '2025-07-31'\n  GROUP BY\n    t1.date\n  ORDER BY\n    t1.date\n  LIMIT 500", "query_result": [{"date": "2025-07-01", "total_daily_reach": 5995346.0}, {"date": "2025-07-02", "total_daily_reach": 6031607.0}, {"date": "2025-07-03", "total_daily_reach": 5917203.0}, {"date": "2025-07-04", "total_daily_reach": 5791901.0}, {"date": "2025-07-05", "total_daily_reach": 5624287.0}, {"date": "2025-07-06", "total_daily_reach": 5629257.0}, {"date": "2025-07-07", "total_daily_reach": 5485384.0}, {"date": "2025-07-08", "total_daily_reach": 5326269.0}, {"date": "2025-07-09", "total_daily_reach": 5230622.0}, {"date": "2025-07-10", "total_daily_reach": 5086002.0}, {"date": "2025-07-11", "total_daily_reach": 4941544.0}, {"date": "2025-07-12", "total_daily_reach": 4788686.0}, {"date": "2025-07-13", "total_daily_reach": 4588218.0}, {"date": "2025-07-14", "total_daily_reach": 4374487.0}, {"date": "2025-07-15", "total_daily_reach": 4287538.0}, {"date": "2025-07-16", "total_daily_reach": 4094771.0}, {"date": "2025-07-17", "total_daily_reach": 4007549.0}, {"date": "2025-07-18", "total_daily_reach": 3767491.0}, {"date": "2025-07-19", "total_daily_reach": 3586414.0}, {"date": "2025-07-20", "total_daily_reach": 3487322.0}, {"date": "2025-07-21", "total_daily_reach": 3237921.0}, {"date": "2025-07-22", "total_daily_reach": 3035686.0}, {"date": "2025-07-23", "total_daily_reach": 2858238.0}, {"date": "2025-07-24", "total_daily_reach": 2634915.0}, {"date": "2025-07-25", "total_daily_reach": 2456400.0}, {"date": "2025-07-26", "total_daily_reach": 2370349.0}, {"date": "2025-07-27", "total_daily_reach": 2094288.0}, {"date": "2025-07-28", "total_daily_reach": 1911266.0}, {"date": "2025-07-29", "total_daily_reach": 3813140.0}, {"date": "2025-07-30", "total_daily_reach": 5533606.0}, {"date": "2025-07-31", "total_daily_reach": 7640471.0}], "db_agent_output": "```json\n{\n  \"explain\": \"The SQL query retrieves the daily reach from the `campaign_performance` table for July 2025. It sums the `reach` for each day and filters the results to include only dates within July 2025. The results are then grouped and ordered by date.\",\n  \"sql\": \"SELECT\\n    t1.date,\\n    SUM(t1.reach) AS total_daily_reach\\n  FROM\\n    `acn-cda.RMN_Campaign_Dataset_Dev.campaign_performance` AS t1\\n  WHERE\\n    t1.date BETWEEN '2025-07-01' AND '2025-07-31'\\n  GROUP BY\\n    t1.date\\n  ORDER BY\\n    t1.date\\n  LIMIT 500\",\n  \"sql_results\": [\n    {\n      \"date\": \"2025-07-01\",\n      \"total_daily_reach\": 5995346\n    },\n    {\n      \"date\": \"2025-07-02\",\n      \"total_daily_reach\": 6031607\n    },\n    {\n      \"date\": \"2025-07-03\",\n      \"total_daily_reach\": 5917203\n    },\n    {\n      \"date\": \"2025-07-04\",\n      \"total_daily_reach\": 5791901\n    },\n    {\n      \"date\": \"2025-07-05\",\n      \"total_daily_reach\": 5624287\n    },\n    {\n      \"date\": \"2025-07-06\",\n      \"total_daily_reach\": 5629257\n    },\n    {\n      \"date\": \"2025-07-07\",\n      \"total_daily_reach\": 5485384\n    },\n    {\n      \"date\": \"2025-07-08\",\n      \"total_daily_reach\": 5326269\n    },\n    {\n      \"date\": \"2025-07-09\",\n      \"total_daily_reach\": 5230622\n    },\n    {\n      \"date\": \"2025-07-10\",\n      \"total_daily_reach\": 5086002\n    },\n    {\n      \"date\": \"2025-07-11\",\n      \"total_daily_reach\": 4941544\n    },\n    {\n      \"date\": \"2025-07-12\",\n      \"total_daily_reach\": 4788686\n    },\n    {\n      \"date\": \"2025-07-13\",\n      \"total_daily_reach\": 4588218\n    },\n    {\n      \"date\": \"2025-07-14\",\n      \"total_daily_reach\": 4374487\n    },\n    {\n      \"date\": \"2025-07-15\",\n      \"total_daily_reach\": 4287538\n    },\n    {\n      \"date\": \"2025-07-16\",\n      \"total_daily_reach\": 4094771\n    },\n    {\n      \"date\": \"2025-07-17\",\n      \"total_daily_reach\": 4007549\n    },\n    {\n      \"date\": \"2025-07-18\",\n      \"total_daily_reach\": 3767491\n    },\n    {\n      \"date\": \"2025-07-19\",\n      \"total_daily_reach\": 3586414\n    },\n    {\n      \"date\": \"2025-07-20\",\n      \"total_daily_reach\": 3487322\n    },\n    {\n      \"date\": \"2025-07-21\",\n      \"total_daily_reach\": 3237921\n    },\n    {\n      \"date\": \"2025-07-22\",\n      \"total_daily_reach\": 3035686\n    },\n    {\n      \"date\": \"2025-07-23\",\n      \"total_daily_reach\": 2858238\n    },\n    {\n      \"date\": \"2025-07-24\",\n      \"total_daily_reach\": 2634915\n    },\n    {\n      \"date\": \"2025-07-25\",\n      \"total_daily_reach\": 2456400\n    },\n    {\n      \"date\": \"2025-07-26\",\n      \"total_daily_reach\": 2370349\n    },\n    {\n      \"date\": \"2025-07-27\",\n      \"total_daily_reach\": 2094288\n    },\n    {\n      \"date\": \"2025-07-28\",\n      \"total_daily_reach\": 1911266\n    },\n    {\n      \"date\": \"2025-07-29\",\n      \"total_daily_reach\": 3813140\n    },\n    {\n      \"date\": \"2025-07-30\",\n      \"total_daily_reach\": 5533606\n    },\n    {\n      \"date\": \"2025-07-31\",\n      \"total_daily_reach\": 7640471\n    }\n  ],\n  \"nl_results\": \"The daily reach for campaigns in July 2025 from the campaign performance table is as follows:\\nJuly 1: 5,995,346\\nJuly 2: 6,031,607\\nJuly 3: 5,917,203\\nJuly 4: 5,791,901\\nJuly 5: 5,624,287\\nJuly 6: 5,629,257\\nJuly 7: 5,485,384\\nJuly 8: 5,326,269\\nJuly 9: 5,230,622\\nJuly 10: 5,086,002\\nJuly 11: 4,941,544\\nJuly 12: 4,788,686\\nJuly 13: 4,588,218\\nJuly 14: 4,374,487\\nJuly 15: 4,287,538\\nJuly 16: 4,094,771\\nJuly 17: 4,007,549\\nJuly 18: 3,767,491\\nJuly 19: 3,586,414\\nJuly 20: 3,487,322\\nJuly 21: 3,237,921\\nJuly 22: 3,035,686\\nJuly 23: 2,858,238\\nJuly 24: 2,634,915\\nJuly 25: 2,456,400\\nJuly 26: 2,370,349\\nJuly 27: 2,094,288\\nJuly 28: 1,911,266\\nJuly 29: 3,813,140\\nJuly 30: 5,533,606\\nJuly 31: 7,640,471\"\n}\n```"}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "x1yZqx0B", "timestamp": 1757660243.889837}, {"content": {"parts": [{"functionCall": {"id": "adk-875a98ee-015b-4585-8ba6-a1df3aa750f4", "args": {"question": "Area chart of daily reach for July 2025."}, "name": "call_viz_agent"}}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7648}], "cachedContentTokenCount": 7648, "candidatesTokenCount": 19, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 19}], "promptTokenCount": 10293, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 10293}], "thoughtsTokenCount": 125, "totalTokenCount": 10437, "trafficType": "ON_DEMAND"}, "invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "longRunningToolIds": [], "id": "T0TSMDfR", "timestamp": 1757660243.891325}, {"content": {"parts": [{"functionResponse": {"id": "adk-875a98ee-015b-4585-8ba6-a1df3aa750f4", "name": "call_viz_agent", "response": {"text": "The area chart visualizes the daily reach for July 2025. It shows a general downward trend in daily reach throughout the month, with a significant increase at the very end of July.", "images": []}}}], "role": "user"}, "invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {"chart_type": "area", "x_axis_label": "Date", "y_axis_label": "Total Daily Reach", "x": [], "y": [], "categories": ["2025-07-01", "2025-07-02", "2025-07-03", "2025-07-04", "2025-07-05", "2025-07-06", "2025-07-07", "2025-07-08", "2025-07-09", "2025-07-10", "2025-07-11", "2025-07-12", "2025-07-13", "2025-07-14", "2025-07-15", "2025-07-16", "2025-07-17", "2025-07-18", "2025-07-19", "2025-07-20", "2025-07-21", "2025-07-22", "2025-07-23", "2025-07-24", "2025-07-25", "2025-07-26", "2025-07-27", "2025-07-28", "2025-07-29", "2025-07-30", "2025-07-31"], "values": [5995346, 6031607, 5917203, 5791901, 5624287, 5629257, 5485384, 5326269, 5230622, 5086002, 4941544, 4788686, 4588218, 4374487, 4287538, 4094771, 4007549, 3767491, 3586414, 3487322, 3237921, 3035686, 2858238, 2634915, 2456400, 2370349, 2094288, 1911266, 3813140, 5533606, 7640471], "title": "Daily Reach for July 2025", "stages": [], "subcategories": [], "dv_agent_output": "The area chart visualizes the daily reach for July 2025. It shows a general downward trend in daily reach throughout the month, with a significant increase at the very end of July."}, "artifactDelta": {"chart_20250912_122742.png": 0}, "requestedAuthConfigs": {}}, "id": "qjdfWhZr", "timestamp": 1757660271.664883}, {"content": {"parts": [{"text": "Result: The area chart visualizes the daily reach for July 2025. It shows a general downward trend in daily reach throughout the month, with a significant increase at the very end of July.\n"}], "role": "model"}, "usageMetadata": {"cacheTokensDetails": [{"modality": "TEXT", "tokenCount": 7631}], "cachedContentTokenCount": 7631, "candidatesTokenCount": 43, "candidatesTokensDetails": [{"modality": "TEXT", "tokenCount": 43}], "promptTokenCount": 10434, "promptTokensDetails": [{"modality": "TEXT", "tokenCount": 10434}], "thoughtsTokenCount": 123, "totalTokenCount": 10600, "trafficType": "ON_DEMAND"}, "invocationId": "e-c1b2e7cd-0311-45be-81b3-2dc0dbc9a1c5", "author": "db_ds_multiagent", "actions": {"stateDelta": {}, "artifactDelta": {}, "requestedAuthConfigs": {}}, "id": "4rR6pjXf", "timestamp": 1757660271.665804}]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:56:39.087850Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2025-09-12T06:57:58.989177Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1:19.901</t>
         </is>
       </c>
     </row>

</xml_diff>